<commit_message>
modified code brfore updated but need some more modification it is not generating time table but accepting new structure
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
+++ b/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00550DE0-6698-4149-A850-98FCC22EF67A}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B958E00-20DE-4454-A36D-4F3EAB78C10E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>faculty name</t>
   </si>
@@ -184,22 +184,28 @@
     <t>Aptitude-2-3</t>
   </si>
   <si>
-    <t>Verbal-2-1</t>
-  </si>
-  <si>
-    <t>verbal-2-2</t>
-  </si>
-  <si>
-    <t>verbal-2-3</t>
-  </si>
-  <si>
     <t>technical-2-3</t>
   </si>
   <si>
     <t>Aptitude-2-4</t>
   </si>
   <si>
-    <t>verbal-2-4</t>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>technical-2-4</t>
+  </si>
+  <si>
+    <t>verbal-2-1</t>
+  </si>
+  <si>
+    <t>Verbal-2-2</t>
+  </si>
+  <si>
+    <t>Verbal-2-3</t>
+  </si>
+  <si>
+    <t>Verbal-2-4</t>
   </si>
 </sst>
 </file>
@@ -566,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B59"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
@@ -975,7 +981,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B51">
         <v>50</v>
@@ -983,7 +989,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B52">
         <v>51</v>
@@ -991,7 +997,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B53">
         <v>52</v>
@@ -999,7 +1005,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B54">
         <v>53</v>
@@ -1007,7 +1013,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B55">
         <v>54</v>
@@ -1015,7 +1021,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56">
         <v>55</v>
@@ -1023,7 +1029,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B57">
         <v>56</v>
@@ -1031,7 +1037,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B58">
         <v>57</v>
@@ -1039,10 +1045,26 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B59">
         <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>56</v>
+      </c>
+      <c r="B60">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes before modification of final one
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
+++ b/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B958E00-20DE-4454-A36D-4F3EAB78C10E}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0B81FC0-25F6-42B2-A615-07A647FFEDAB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>faculty name</t>
   </si>
@@ -206,6 +206,12 @@
   </si>
   <si>
     <t>Verbal-2-4</t>
+  </si>
+  <si>
+    <t>verbal-3 year</t>
+  </si>
+  <si>
+    <t>aptitude-3 year</t>
   </si>
 </sst>
 </file>
@@ -572,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
@@ -1067,6 +1073,22 @@
         <v>60</v>
       </c>
     </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B42">
     <sortCondition ref="A1:A42"/>

</xml_diff>

<commit_message>
updates till before holidays
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
+++ b/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0B81FC0-25F6-42B2-A615-07A647FFEDAB}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB492733-F183-49EE-BB0D-394226A3C10E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
   <si>
     <t>faculty name</t>
   </si>
@@ -202,23 +202,86 @@
     <t>Verbal-2-2</t>
   </si>
   <si>
-    <t>Verbal-2-3</t>
-  </si>
-  <si>
-    <t>Verbal-2-4</t>
-  </si>
-  <si>
     <t>verbal-3 year</t>
   </si>
   <si>
     <t>aptitude-3 year</t>
+  </si>
+  <si>
+    <t>technical-2-5</t>
+  </si>
+  <si>
+    <t>technical-2-6</t>
+  </si>
+  <si>
+    <t>technical-2-7</t>
+  </si>
+  <si>
+    <t>technical-2-8</t>
+  </si>
+  <si>
+    <t>technical-2-9</t>
+  </si>
+  <si>
+    <t>technical-2-10</t>
+  </si>
+  <si>
+    <t>technical-2-11</t>
+  </si>
+  <si>
+    <t>Aptitude-2-5</t>
+  </si>
+  <si>
+    <t>Aptitude-2-6</t>
+  </si>
+  <si>
+    <t>Aptitude-2-7</t>
+  </si>
+  <si>
+    <t>Aptitude-2-8</t>
+  </si>
+  <si>
+    <t>Aptitude-2-9</t>
+  </si>
+  <si>
+    <t>Aptitude-2-10</t>
+  </si>
+  <si>
+    <t>Aptitude-2-11</t>
+  </si>
+  <si>
+    <t>verbal-2-3</t>
+  </si>
+  <si>
+    <t>verbal-2-4</t>
+  </si>
+  <si>
+    <t>verbal-2-5</t>
+  </si>
+  <si>
+    <t>verbal-2-6</t>
+  </si>
+  <si>
+    <t>verbal-2-7</t>
+  </si>
+  <si>
+    <t>verbal-2-8</t>
+  </si>
+  <si>
+    <t>verbal-2-9</t>
+  </si>
+  <si>
+    <t>verbal-2-10</t>
+  </si>
+  <si>
+    <t>verbal-2-11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,6 +293,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -578,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
@@ -995,7 +1064,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B52">
         <v>51</v>
@@ -1003,7 +1072,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B53">
         <v>52</v>
@@ -1011,7 +1080,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B54">
         <v>53</v>
@@ -1019,7 +1088,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B55">
         <v>54</v>
@@ -1027,7 +1096,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B56">
         <v>55</v>
@@ -1035,7 +1104,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B57">
         <v>56</v>
@@ -1043,7 +1112,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B58">
         <v>57</v>
@@ -1051,7 +1120,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B59">
         <v>58</v>
@@ -1059,7 +1128,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B60">
         <v>59</v>
@@ -1067,7 +1136,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B61">
         <v>60</v>
@@ -1075,7 +1144,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B62">
         <v>61</v>
@@ -1083,16 +1152,193 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B63">
         <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>55</v>
+      </c>
+      <c r="B64">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>72</v>
+      </c>
+      <c r="B68">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>73</v>
+      </c>
+      <c r="B69">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>75</v>
+      </c>
+      <c r="B71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>58</v>
+      </c>
+      <c r="B72">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>56</v>
+      </c>
+      <c r="B83">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>60</v>
+      </c>
+      <c r="B84">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>61</v>
+      </c>
+      <c r="B85">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B42">
     <sortCondition ref="A1:A42"/>
   </sortState>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
all updated input files
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
+++ b/TIME TABLE SAMPLE DATA/FACULTY ID MAPPING.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ganig\Desktop\Time_Table_\TIME TABLE SAMPLE DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="166" documentId="11_2B59D2BFD3605E4F694397735B3088B352998C3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB492733-F183-49EE-BB0D-394226A3C10E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D230CF94-8C6E-470F-9676-E2A44436EF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>faculty name</t>
   </si>
@@ -151,130 +151,7 @@
     <t>D.Venkata Reddy</t>
   </si>
   <si>
-    <t>kiran---aptitude</t>
-  </si>
-  <si>
-    <t>janaki---vebal</t>
-  </si>
-  <si>
-    <t>mern</t>
-  </si>
-  <si>
-    <t>da</t>
-  </si>
-  <si>
-    <t>java</t>
-  </si>
-  <si>
-    <t>technical---3year</t>
-  </si>
-  <si>
-    <t>technical-2-1</t>
-  </si>
-  <si>
-    <t>technical-2-2</t>
-  </si>
-  <si>
-    <t>Aptitude-2-1</t>
-  </si>
-  <si>
-    <t>Aptitude-2-2</t>
-  </si>
-  <si>
-    <t>Aptitude-2-3</t>
-  </si>
-  <si>
-    <t>technical-2-3</t>
-  </si>
-  <si>
-    <t>Aptitude-2-4</t>
-  </si>
-  <si>
     <t>PT</t>
-  </si>
-  <si>
-    <t>technical-2-4</t>
-  </si>
-  <si>
-    <t>verbal-2-1</t>
-  </si>
-  <si>
-    <t>Verbal-2-2</t>
-  </si>
-  <si>
-    <t>verbal-3 year</t>
-  </si>
-  <si>
-    <t>aptitude-3 year</t>
-  </si>
-  <si>
-    <t>technical-2-5</t>
-  </si>
-  <si>
-    <t>technical-2-6</t>
-  </si>
-  <si>
-    <t>technical-2-7</t>
-  </si>
-  <si>
-    <t>technical-2-8</t>
-  </si>
-  <si>
-    <t>technical-2-9</t>
-  </si>
-  <si>
-    <t>technical-2-10</t>
-  </si>
-  <si>
-    <t>technical-2-11</t>
-  </si>
-  <si>
-    <t>Aptitude-2-5</t>
-  </si>
-  <si>
-    <t>Aptitude-2-6</t>
-  </si>
-  <si>
-    <t>Aptitude-2-7</t>
-  </si>
-  <si>
-    <t>Aptitude-2-8</t>
-  </si>
-  <si>
-    <t>Aptitude-2-9</t>
-  </si>
-  <si>
-    <t>Aptitude-2-10</t>
-  </si>
-  <si>
-    <t>Aptitude-2-11</t>
-  </si>
-  <si>
-    <t>verbal-2-3</t>
-  </si>
-  <si>
-    <t>verbal-2-4</t>
-  </si>
-  <si>
-    <t>verbal-2-5</t>
-  </si>
-  <si>
-    <t>verbal-2-6</t>
-  </si>
-  <si>
-    <t>verbal-2-7</t>
-  </si>
-  <si>
-    <t>verbal-2-8</t>
-  </si>
-  <si>
-    <t>verbal-2-9</t>
-  </si>
-  <si>
-    <t>verbal-2-10</t>
-  </si>
-  <si>
-    <t>verbal-2-11</t>
   </si>
 </sst>
 </file>
@@ -356,10 +233,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -647,14 +520,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B85"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B43"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -662,7 +535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -670,7 +543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -678,7 +551,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -686,7 +559,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -694,7 +567,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -702,7 +575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -710,7 +583,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -718,7 +591,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -726,7 +599,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -734,7 +607,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -742,7 +615,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -750,7 +623,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -758,7 +631,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -766,7 +639,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -774,7 +647,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -782,7 +655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -790,7 +663,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -798,7 +671,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -806,7 +679,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -814,7 +687,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -822,7 +695,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -830,7 +703,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -838,7 +711,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>41</v>
       </c>
@@ -846,7 +719,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -854,7 +727,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -862,7 +735,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -870,7 +743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -878,7 +751,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>6</v>
       </c>
@@ -886,7 +759,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -894,7 +767,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -902,7 +775,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>17</v>
       </c>
@@ -910,7 +783,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -918,7 +791,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -926,7 +799,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -934,7 +807,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -942,7 +815,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -950,7 +823,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -958,7 +831,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -966,7 +839,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>20</v>
       </c>
@@ -974,7 +847,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -982,7 +855,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -990,348 +863,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>43</v>
       </c>
       <c r="B43">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>47</v>
-      </c>
-      <c r="B47">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>50</v>
-      </c>
-      <c r="B50">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>54</v>
-      </c>
-      <c r="B52">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>57</v>
-      </c>
-      <c r="B53">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>62</v>
-      </c>
-      <c r="B54">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>63</v>
-      </c>
-      <c r="B55">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>64</v>
-      </c>
-      <c r="B56">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>65</v>
-      </c>
-      <c r="B57">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>66</v>
-      </c>
-      <c r="B58">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>67</v>
-      </c>
-      <c r="B59">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>68</v>
-      </c>
-      <c r="B60">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>51</v>
-      </c>
-      <c r="B61">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>53</v>
-      </c>
-      <c r="B63">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>55</v>
-      </c>
-      <c r="B64">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>69</v>
-      </c>
-      <c r="B65">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>70</v>
-      </c>
-      <c r="B66">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>71</v>
-      </c>
-      <c r="B67">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>73</v>
-      </c>
-      <c r="B69">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>74</v>
-      </c>
-      <c r="B70">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>75</v>
-      </c>
-      <c r="B71">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>58</v>
-      </c>
-      <c r="B72">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>59</v>
-      </c>
-      <c r="B73">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>76</v>
-      </c>
-      <c r="B74">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>77</v>
-      </c>
-      <c r="B75">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>78</v>
-      </c>
-      <c r="B76">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>79</v>
-      </c>
-      <c r="B77">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>80</v>
-      </c>
-      <c r="B78">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>81</v>
-      </c>
-      <c r="B79">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
         <v>82</v>
-      </c>
-      <c r="B80">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>83</v>
-      </c>
-      <c r="B81">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>84</v>
-      </c>
-      <c r="B82">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>56</v>
-      </c>
-      <c r="B83">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>60</v>
-      </c>
-      <c r="B84">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>61</v>
-      </c>
-      <c r="B85">
-        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>